<commit_message>
S7 Table: discovery cohort 856 lines (22 same-patient models excluded), sheet name, low-n flag column name
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/figures/supporting_information/S7_Table.xlsx
+++ b/figures/supporting_information/S7_Table.xlsx
@@ -441,14 +441,14 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Discovery cohort: the 878 DepMap 26Q1 cancer cell lines without any Sanger (KY-library) screen in the combined 26Q1 data set; the complete procedure (one-sided Mann-Whitney, BH over all tests, q &lt; 0.05, median Chronos &lt; -1, selectivity &lt; -0.5) was applied to it.</t>
+          <t>Discovery cohort: the 856 DepMap 26Q1 cancer cell lines without any Sanger (KY-library) screen in the combined 26Q1 data set, after excluding 22 models derived from the same patient as a Project Score model; the complete procedure (one-sided Mann-Whitney, BH over all tests, q &lt; 0.05, median Chronos &lt; -1, selectivity &lt; -0.5) was applied to it.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Replication: the same procedure applied to the Sanger Project Score Chronos data (316 cancer models); discovery and replication share no screens and no cell lines.</t>
+          <t>Replication: the same procedure applied to the Sanger Project Score Chronos data (316 cancer models); discovery and replication share no screens, models or patients.</t>
         </is>
       </c>
     </row>
@@ -462,7 +462,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Sheet 'Overlapping comparison (not independent)': earlier comparison of the primary candidates with the Sanger data. For the shared cell lines the 26Q1 gene effects include the same Sanger screens, so this comparison is not independent; shown for transparency only.</t>
+          <t>Sheet 'Overlapping (not independent)': earlier comparison of the primary candidates with the Sanger data. For the shared cell lines the 26Q1 gene effects include the same Sanger screens, so this comparison is not independent; shown for transparency only.</t>
         </is>
       </c>
     </row>
@@ -9331,7 +9331,7 @@
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>confidence</t>
+          <t>Low-n flag (fewer than 10 target lines)</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">

</xml_diff>